<commit_message>
feat(invoice-extract): strict Taskforce parse, exact address match, A–J Excel row
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/lib/invoice-templates/taskforce/template.xlsx
+++ b/lib/invoice-templates/taskforce/template.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Invoices" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Ledger</t>
   </si>
@@ -22,7 +22,7 @@
     <t>GST Code</t>
   </si>
   <si>
-    <t>Amount (Inc GST)</t>
+    <t>Amount</t>
   </si>
   <si>
     <t>Service</t>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t>Account number from RTA property list</t>
+  </si>
+  <si>
+    <t>Notes</t>
   </si>
 </sst>
 </file>
@@ -414,21 +417,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="40" customWidth="1"/>
-    <col min="6" max="6" width="45" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="6" width="48" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="36" customWidth="1"/>
+    <col min="9" max="9" width="40" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -455,6 +458,9 @@
       </c>
       <c r="I1" t="s">
         <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>